<commit_message>
Working bot before adding conversation memory
</commit_message>
<xml_diff>
--- a/data/price-sheet.xlsx
+++ b/data/price-sheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OMEN GAMING\Documents\fabian\trial-price-sheet-chatbot (2)\trial-price-sheet-chatbot\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OMEN GAMING\Documents\fabian\projects\maxmed-bot\maxmed-bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F23ADC1A-63C2-4A63-81B8-8D7162F37CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9E022F-6E86-44AC-868B-1108B1E127A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Strips" sheetId="1" r:id="rId1"/>
@@ -550,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -578,13 +578,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -596,21 +596,33 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -620,7 +632,10 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -629,31 +644,19 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -977,7 +980,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1009,10 +1012,10 @@
       <c r="D2" s="4">
         <v>40</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="37">
         <v>25</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="12" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="5" t="s">
@@ -1035,7 +1038,7 @@
       <c r="E3" s="4">
         <v>15</v>
       </c>
-      <c r="F3" s="12"/>
+      <c r="F3" s="13"/>
       <c r="G3" s="5" t="s">
         <v>9</v>
       </c>
@@ -1056,13 +1059,13 @@
       <c r="E4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="12"/>
+      <c r="F4" s="13"/>
       <c r="G4" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F5" s="12"/>
+      <c r="F5" s="13"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -1080,7 +1083,7 @@
       <c r="E6" s="4">
         <v>8</v>
       </c>
-      <c r="F6" s="12"/>
+      <c r="F6" s="13"/>
       <c r="G6" s="5" t="s">
         <v>9</v>
       </c>
@@ -1101,7 +1104,7 @@
       <c r="E7" s="4">
         <v>4</v>
       </c>
-      <c r="F7" s="12"/>
+      <c r="F7" s="13"/>
       <c r="G7" s="5" t="s">
         <v>9</v>
       </c>
@@ -1122,13 +1125,13 @@
       <c r="E8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="12"/>
+      <c r="F8" s="13"/>
       <c r="G8" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F9" s="12"/>
+      <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -1146,7 +1149,7 @@
       <c r="E10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="12"/>
+      <c r="F10" s="13"/>
       <c r="G10" s="5" t="s">
         <v>9</v>
       </c>
@@ -1167,13 +1170,13 @@
       <c r="E11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="12"/>
+      <c r="F11" s="13"/>
       <c r="G11" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F12" s="12"/>
+      <c r="F12" s="13"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -1191,7 +1194,7 @@
       <c r="E13" s="4">
         <v>25</v>
       </c>
-      <c r="F13" s="12"/>
+      <c r="F13" s="13"/>
       <c r="G13" s="5" t="s">
         <v>9</v>
       </c>
@@ -1212,7 +1215,7 @@
       <c r="E14" s="4">
         <v>15</v>
       </c>
-      <c r="F14" s="12"/>
+      <c r="F14" s="13"/>
       <c r="G14" s="5" t="s">
         <v>9</v>
       </c>
@@ -1233,7 +1236,7 @@
       <c r="E15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F15" s="12"/>
+      <c r="F15" s="13"/>
       <c r="G15" s="5" t="s">
         <v>9</v>
       </c>
@@ -1254,7 +1257,7 @@
       <c r="E16" s="4">
         <v>20</v>
       </c>
-      <c r="F16" s="12"/>
+      <c r="F16" s="13"/>
       <c r="G16" s="5" t="s">
         <v>9</v>
       </c>
@@ -1275,7 +1278,7 @@
       <c r="E17" s="4">
         <v>8</v>
       </c>
-      <c r="F17" s="12"/>
+      <c r="F17" s="13"/>
       <c r="G17" s="5" t="s">
         <v>9</v>
       </c>
@@ -1296,13 +1299,13 @@
       <c r="E18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="12"/>
+      <c r="F18" s="13"/>
       <c r="G18" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F19" s="12"/>
+      <c r="F19" s="13"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
@@ -1320,7 +1323,7 @@
       <c r="E20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F20" s="12"/>
+      <c r="F20" s="13"/>
       <c r="G20" s="5" t="s">
         <v>9</v>
       </c>
@@ -1341,7 +1344,7 @@
       <c r="E21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F21" s="12"/>
+      <c r="F21" s="13"/>
       <c r="G21" s="5" t="s">
         <v>9</v>
       </c>
@@ -1362,7 +1365,7 @@
       <c r="E22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="12"/>
+      <c r="F22" s="13"/>
       <c r="G22" s="5" t="s">
         <v>9</v>
       </c>
@@ -1383,7 +1386,7 @@
       <c r="E23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F23" s="12"/>
+      <c r="F23" s="13"/>
       <c r="G23" s="5" t="s">
         <v>9</v>
       </c>
@@ -1404,7 +1407,7 @@
       <c r="E24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F24" s="12"/>
+      <c r="F24" s="13"/>
       <c r="G24" s="5" t="s">
         <v>9</v>
       </c>
@@ -1425,7 +1428,7 @@
       <c r="E25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F25" s="12"/>
+      <c r="F25" s="13"/>
       <c r="G25" s="5" t="s">
         <v>9</v>
       </c>
@@ -1446,7 +1449,7 @@
       <c r="E26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F26" s="12"/>
+      <c r="F26" s="13"/>
       <c r="G26" s="5" t="s">
         <v>9</v>
       </c>
@@ -1467,7 +1470,7 @@
       <c r="E27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F27" s="12"/>
+      <c r="F27" s="13"/>
       <c r="G27" s="5" t="s">
         <v>9</v>
       </c>
@@ -1476,7 +1479,7 @@
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="11" t="s">
         <v>31</v>
       </c>
       <c r="C29" s="14"/>
@@ -1496,12 +1499,12 @@
       <c r="B30" s="4">
         <v>40</v>
       </c>
-      <c r="C30" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="11" t="s">
+      <c r="C30" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="12" t="s">
         <v>8</v>
       </c>
       <c r="G30" s="5" t="s">
@@ -1515,10 +1518,10 @@
       <c r="B31" s="4">
         <v>10</v>
       </c>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="12"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="13"/>
       <c r="G31" s="5" t="s">
         <v>9</v>
       </c>
@@ -1530,10 +1533,10 @@
       <c r="B32" s="4">
         <v>10</v>
       </c>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="12"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="13"/>
       <c r="G32" s="5" t="s">
         <v>9</v>
       </c>
@@ -1545,19 +1548,19 @@
       <c r="B33" s="4">
         <v>5</v>
       </c>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="12"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="13"/>
       <c r="G33" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="12"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="13"/>
     </row>
     <row r="35" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
@@ -1566,10 +1569,10 @@
       <c r="B35" s="4">
         <v>20</v>
       </c>
-      <c r="C35" s="33"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="12"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="13"/>
       <c r="G35" s="5" t="s">
         <v>9</v>
       </c>
@@ -1581,10 +1584,10 @@
       <c r="B36" s="4">
         <v>10</v>
       </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="12"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="13"/>
       <c r="G36" s="5" t="s">
         <v>9</v>
       </c>
@@ -1596,10 +1599,10 @@
       <c r="B37" s="4">
         <v>10</v>
       </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="12"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="13"/>
       <c r="G37" s="5" t="s">
         <v>9</v>
       </c>
@@ -1611,10 +1614,10 @@
       <c r="B38" s="4">
         <v>5</v>
       </c>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="12"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="13"/>
       <c r="G38" s="5" t="s">
         <v>9</v>
       </c>
@@ -1627,6 +1630,7 @@
     <mergeCell ref="F30:F38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1686,7 +1690,7 @@
       <c r="F2" s="4">
         <v>150</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="21" t="s">
         <v>48</v>
       </c>
       <c r="H2" s="5">
@@ -1712,7 +1716,7 @@
       <c r="F3" s="4">
         <v>150</v>
       </c>
-      <c r="G3" s="18"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="5">
         <v>150</v>
       </c>
@@ -1736,7 +1740,7 @@
       <c r="F4" s="4">
         <v>100</v>
       </c>
-      <c r="G4" s="18"/>
+      <c r="G4" s="22"/>
       <c r="H4" s="5">
         <v>150</v>
       </c>
@@ -1760,7 +1764,7 @@
       <c r="F5" s="4">
         <v>100</v>
       </c>
-      <c r="G5" s="18"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="5">
         <v>150</v>
       </c>
@@ -1784,7 +1788,7 @@
       <c r="F6" s="4">
         <v>25</v>
       </c>
-      <c r="G6" s="18"/>
+      <c r="G6" s="22"/>
       <c r="H6" s="5">
         <v>25</v>
       </c>
@@ -1808,21 +1812,21 @@
       <c r="F7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="18"/>
+      <c r="G7" s="22"/>
       <c r="H7" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
       <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1835,12 +1839,12 @@
       <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="19" t="s">
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="30" t="s">
         <v>57</v>
       </c>
       <c r="H9" s="5"/>
@@ -1855,10 +1859,10 @@
       <c r="C10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="12"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="13"/>
       <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -1871,10 +1875,10 @@
       <c r="C11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="12"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="13"/>
       <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1887,10 +1891,10 @@
       <c r="C12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="12"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="13"/>
       <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1912,7 +1916,7 @@
       <c r="F13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="30" t="s">
         <v>90</v>
       </c>
       <c r="H13" s="5">
@@ -1938,7 +1942,7 @@
       <c r="F14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="12"/>
+      <c r="G14" s="13"/>
       <c r="H14" s="5" t="s">
         <v>9</v>
       </c>
@@ -1962,7 +1966,7 @@
       <c r="F15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="12"/>
+      <c r="G15" s="13"/>
       <c r="H15" s="5" t="s">
         <v>9</v>
       </c>
@@ -2012,7 +2016,7 @@
       <c r="F17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="21" t="s">
         <v>67</v>
       </c>
       <c r="H17" s="5">
@@ -2038,7 +2042,7 @@
       <c r="F18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="18"/>
+      <c r="G18" s="22"/>
       <c r="H18" s="5">
         <v>50</v>
       </c>
@@ -2062,7 +2066,7 @@
       <c r="F19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G19" s="18"/>
+      <c r="G19" s="22"/>
       <c r="H19" s="5">
         <v>50</v>
       </c>
@@ -2086,7 +2090,7 @@
       <c r="F20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="18"/>
+      <c r="G20" s="22"/>
       <c r="H20" s="5">
         <v>50</v>
       </c>
@@ -2110,7 +2114,7 @@
       <c r="F21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G21" s="18"/>
+      <c r="G21" s="22"/>
       <c r="H21" s="5">
         <v>50</v>
       </c>
@@ -2134,7 +2138,7 @@
       <c r="F22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="18"/>
+      <c r="G22" s="22"/>
       <c r="H22" s="5">
         <v>50</v>
       </c>
@@ -2158,7 +2162,7 @@
       <c r="F23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G23" s="18"/>
+      <c r="G23" s="22"/>
       <c r="H23" s="5">
         <v>50</v>
       </c>
@@ -2182,7 +2186,7 @@
       <c r="F24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="18"/>
+      <c r="G24" s="22"/>
       <c r="H24" s="5">
         <v>20</v>
       </c>
@@ -2206,21 +2210,21 @@
       <c r="F25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="28"/>
+      <c r="G25" s="23"/>
       <c r="H25" s="5">
         <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
       <c r="H26" s="5"/>
     </row>
     <row r="27" spans="1:8" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2233,12 +2237,12 @@
       <c r="C27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="22" t="s">
+      <c r="D27" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="29" t="s">
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="24" t="s">
         <v>74</v>
       </c>
       <c r="H27" s="5" t="s">
@@ -2255,10 +2259,10 @@
       <c r="C28" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="30"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="25"/>
       <c r="H28" s="5" t="s">
         <v>9</v>
       </c>
@@ -2273,10 +2277,10 @@
       <c r="C29" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="30"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="25"/>
       <c r="H29" s="5" t="s">
         <v>9</v>
       </c>
@@ -2336,7 +2340,7 @@
       <c r="C2" s="4">
         <v>5</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="21" t="s">
         <v>80</v>
       </c>
       <c r="E2" s="5">
@@ -2353,7 +2357,7 @@
       <c r="C3" s="4">
         <v>5</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="22"/>
       <c r="E3" s="5">
         <v>35</v>
       </c>
@@ -2368,7 +2372,7 @@
       <c r="C4" s="4">
         <v>5</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="22"/>
       <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -2381,7 +2385,7 @@
       <c r="C5" s="4">
         <v>5</v>
       </c>
-      <c r="D5" s="18"/>
+      <c r="D5" s="22"/>
       <c r="E5" s="5">
         <v>25</v>
       </c>
@@ -2396,7 +2400,7 @@
       <c r="C6" s="4">
         <v>5</v>
       </c>
-      <c r="D6" s="18"/>
+      <c r="D6" s="22"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -2409,7 +2413,7 @@
       <c r="C7" s="4">
         <v>5</v>
       </c>
-      <c r="D7" s="28"/>
+      <c r="D7" s="23"/>
       <c r="E7" s="5">
         <v>25</v>
       </c>
@@ -2421,10 +2425,10 @@
       <c r="B8" s="4">
         <v>50</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="32"/>
+      <c r="D8" s="34"/>
       <c r="E8" s="5">
         <v>25</v>
       </c>
@@ -2436,8 +2440,8 @@
       <c r="B9" s="4">
         <v>50</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="34"/>
       <c r="E9" s="5">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
Final: disambiguation fix for Dexcom + all features working (230+ tests)
</commit_message>
<xml_diff>
--- a/data/price-sheet.xlsx
+++ b/data/price-sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OMEN GAMING\Documents\fabian\projects\maxmed-bot\maxmed-bot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9E022F-6E86-44AC-868B-1108B1E127A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39420BB3-835B-41B9-BED9-E5519A932B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Strips" sheetId="1" r:id="rId1"/>
@@ -550,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -654,9 +654,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1012,7 +1009,7 @@
       <c r="D2" s="4">
         <v>40</v>
       </c>
-      <c r="E2" s="37">
+      <c r="E2" s="4">
         <v>25</v>
       </c>
       <c r="F2" s="12" t="s">

</xml_diff>